<commit_message>
Add employee robot greeting and attendance history filters
Welcome employees once daily with speech-completion dismissal, add attendance filters and start/end distances, center dark Excel headers, and remove automatic non-billable activity annotations.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/geosite/excel_templates/activity_report.xlsx
+++ b/geosite/excel_templates/activity_report.xlsx
@@ -200,7 +200,7 @@
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -232,7 +232,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>

</xml_diff>